<commit_message>
zipcode-gate-login: employer-sponsored FAQ as an accordion
The source's "What is employer-sponsored health insurance?" is a one-item
FAQ accordion (collapsed by default), the same markup as the
/resources/answers/faq pages. Map it to accordion-minimal-light and reuse
that block's parser instead of flattening it into a bold question and an
answer paragraph. Re-imported, uploaded to DA and previewed.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-zipcode-gate-login.report.xlsx
+++ b/tools/importer/reports/import-zipcode-gate-login.report.xlsx
@@ -283,13 +283,13 @@
     <t>zipcode-gate-login.report.json</t>
   </si>
   <si>
-    <t>["zip-county-form"]</t>
+    <t>["zip-county-form","accordion-minimal-light"]</t>
   </si>
   <si>
     <t>zipcode-gate-login</t>
   </si>
   <si>
-    <t>2026-10-05T16:34:47.859Z</t>
+    <t>2026-10-06T11:01:05.594Z</t>
   </si>
   <si>
     <t>https://www.highmark.com/zipcode-gate-login</t>

</xml_diff>